<commit_message>
Add --ignore "sheetName:regex" to supress diff messages
all differences in the LINE of "sheetName" that contains "regex" in the NEW values, will not be reported.

Useful for filtering out messages that include today's date, git hashes, etc.
</commit_message>
<xml_diff>
--- a/test_data/xlsx_diff/new.xlsx
+++ b/test_data/xlsx_diff/new.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/curtish/Documents/ICTV/ICTVvmrUpdate/test_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/curtish/Documents/ICTV/ICTVvmr-update/test_data/xlsx_diff/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{463193D6-9289-7F48-9A2E-7AD0CFDBDAE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49083EC1-23D8-EB46-98A8-F7DCD7C40F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3340" yWindow="3660" windowWidth="25640" windowHeight="14440" xr2:uid="{295F2116-0CB0-C048-85BD-FF48A684A5E6}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>june</t>
   </si>
@@ -46,6 +46,15 @@
   </si>
   <si>
     <t>ernie</t>
+  </si>
+  <si>
+    <t>real difference</t>
+  </si>
+  <si>
+    <t>and this will not be seen either</t>
+  </si>
+  <si>
+    <t>ignore this line</t>
   </si>
 </sst>
 </file>
@@ -417,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2041A03-887F-474F-AA34-B33A16095E0E}">
-  <dimension ref="A2:C3"/>
+  <dimension ref="A2:C7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -431,6 +440,19 @@
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>